<commit_message>
Align forestry reports with B.1-B.7 and add forest land cross-tab
</commit_message>
<xml_diff>
--- a/skills/forestry-survey-summary-tables/assets/report-headers.xlsx
+++ b/skills/forestry-survey-summary-tables/assets/report-headers.xlsx
@@ -8,21 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Finn\Documents\GitHub\agent-skills\skills\forestry-survey-summary-tables\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAEA0E98-1DE8-4BDF-9921-3822E416D5C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DACD0C77-0F80-4225-94BB-E4926C61F13B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7200" yWindow="4610" windowWidth="21600" windowHeight="12670" xr2:uid="{6C185909-5B95-4627-AE85-729272F08AC2}"/>
+    <workbookView xWindow="4520" yWindow="4520" windowWidth="21600" windowHeight="12670" xr2:uid="{6C185909-5B95-4627-AE85-729272F08AC2}"/>
   </bookViews>
   <sheets>
-    <sheet name="1" sheetId="2" r:id="rId1"/>
-    <sheet name="2" sheetId="3" r:id="rId2"/>
-    <sheet name="3" sheetId="4" r:id="rId3"/>
-    <sheet name="4" sheetId="5" r:id="rId4"/>
-    <sheet name="5" sheetId="6" r:id="rId5"/>
-    <sheet name="6" sheetId="8" r:id="rId6"/>
-    <sheet name="7" sheetId="7" r:id="rId7"/>
+    <sheet name="B.1" sheetId="2" r:id="rId1"/>
+    <sheet name="B.2" sheetId="3" r:id="rId2"/>
+    <sheet name="B.3" sheetId="4" r:id="rId3"/>
+    <sheet name="B.4" sheetId="5" r:id="rId4"/>
+    <sheet name="B.5" sheetId="9" r:id="rId5"/>
+    <sheet name="B.6" sheetId="6" r:id="rId6"/>
+    <sheet name="B.7" sheetId="8" r:id="rId7"/>
+    <sheet name="小班明细" sheetId="7" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'6'!$A$1:$AB$7</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">B.5!$A$1:$O$6</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">B.7!$A$1:$AB$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">B.5!$1:$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="99">
   <si>
     <t>单位：公顷、立方米</t>
   </si>
@@ -103,10 +106,6 @@
 林地</t>
   </si>
   <si>
-    <t>附表1</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>现  状  地  类</t>
   </si>
   <si>
@@ -140,10 +139,6 @@
 迹地</t>
   </si>
   <si>
-    <t>附表2</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>森  林  类  别</t>
   </si>
   <si>
@@ -183,10 +178,6 @@
     <t>三级</t>
   </si>
   <si>
-    <t>附表3</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>单位：公顷</t>
   </si>
   <si>
@@ -205,10 +196,6 @@
     <t>Ⅳ级</t>
   </si>
   <si>
-    <t>附表4</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>重点生态区域名称</t>
   </si>
   <si>
@@ -234,10 +221,6 @@
   </si>
   <si>
     <t>面积</t>
-  </si>
-  <si>
-    <t>附表5</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>县</t>
@@ -389,39 +372,76 @@
 性质</t>
   </si>
   <si>
-    <t>附表7</t>
+    <t>单位：公顷、元/平方米、万元</t>
+  </si>
+  <si>
+    <t>总计</t>
+  </si>
+  <si>
+    <t>乔木林地(含迹地)</t>
+  </si>
+  <si>
+    <t>天然林</t>
+  </si>
+  <si>
+    <t>人工林及其它</t>
+  </si>
+  <si>
+    <t>灌木林地</t>
+  </si>
+  <si>
+    <t>其他无立木林地</t>
+  </si>
+  <si>
+    <t>恢复费</t>
+  </si>
+  <si>
+    <t>标准</t>
+  </si>
+  <si>
+    <t>表B.1</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>单位：公顷、元/平方米、万元</t>
-  </si>
-  <si>
-    <t>总计</t>
-  </si>
-  <si>
-    <t>乔木林地(含迹地)</t>
-  </si>
-  <si>
-    <t>天然林</t>
-  </si>
-  <si>
-    <t>人工林及其它</t>
-  </si>
-  <si>
-    <t>灌木林地</t>
-  </si>
-  <si>
-    <t>其他无立木林地</t>
-  </si>
-  <si>
-    <t>恢复费</t>
-  </si>
-  <si>
-    <t>标准</t>
-  </si>
-  <si>
-    <t>附表6 使用林地森林植被恢复费测算表</t>
+    <t>表B.2</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>表B.3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>表B.4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>表B.6</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>表B.7 使用林地森林植被恢复费测算表</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>表B.5 项目使用林地分森林类别按地类面积统计表</t>
+  </si>
+  <si>
+    <t>国有</t>
+  </si>
+  <si>
+    <t>集体</t>
+  </si>
+  <si>
+    <t>乔木林地</t>
+  </si>
+  <si>
+    <t>国家特别规定灌木林地</t>
+  </si>
+  <si>
+    <t>一般灌木林地</t>
   </si>
 </sst>
 </file>
@@ -434,7 +454,7 @@
     <numFmt numFmtId="178" formatCode="0_ "/>
     <numFmt numFmtId="179" formatCode="0.00_ "/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -491,6 +511,21 @@
       <name val="宋体"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -538,7 +573,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -575,40 +610,52 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="177" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="177" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -942,7 +989,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>16</v>
+        <v>86</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -985,50 +1032,50 @@
       <c r="H3" s="2"/>
       <c r="I3" s="2"/>
       <c r="J3" s="2"/>
-      <c r="K3" s="21" t="s">
+      <c r="K3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="L3" s="21"/>
-      <c r="M3" s="21"/>
-      <c r="N3" s="21"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
     </row>
     <row r="4" spans="1:14" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
     </row>
     <row r="5" spans="1:14" ht="30.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
       <c r="G5" s="3" t="s">
         <v>8</v>
       </c>
@@ -1088,7 +1135,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>26</v>
+        <v>87</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1140,82 +1187,82 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
-      <c r="N3" s="21" t="s">
+      <c r="N3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21"/>
-      <c r="Q3" s="21"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
     </row>
     <row r="4" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
+      <c r="G4" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
     </row>
     <row r="5" spans="1:17" ht="30.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
       <c r="G5" s="3" t="s">
         <v>8</v>
       </c>
       <c r="H5" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="I5" s="3" t="s">
+      <c r="J5" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="J5" s="3" t="s">
+      <c r="K5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="3" t="s">
+      <c r="M5" s="3" t="s">
         <v>22</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="N5" s="3" t="s">
         <v>14</v>
       </c>
       <c r="O5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="P5" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="P5" s="3" t="s">
-        <v>25</v>
       </c>
       <c r="Q5" s="3" t="s">
         <v>15</v>
@@ -1259,7 +1306,7 @@
   <sheetData>
     <row r="1" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1311,133 +1358,136 @@
       <c r="K3" s="2"/>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
-      <c r="N3" s="21" t="s">
+      <c r="N3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="O3" s="21"/>
-      <c r="P3" s="21"/>
-      <c r="Q3" s="21"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
     </row>
     <row r="4" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+    </row>
+    <row r="5" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
-    </row>
-    <row r="5" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="16" t="s">
-        <v>8</v>
-      </c>
-      <c r="H5" s="16" t="s">
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+    </row>
+    <row r="6" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="16" t="s">
+      <c r="I6" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-    </row>
-    <row r="6" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="18" t="s">
+      <c r="J6" s="18"/>
+      <c r="K6" s="18"/>
+      <c r="L6" s="18"/>
+      <c r="M6" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="I6" s="16" t="s">
+      <c r="N6" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="J6" s="22"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="22"/>
-      <c r="M6" s="18" t="s">
+      <c r="O6" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="P6" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="N6" s="18" t="s">
+      <c r="Q6" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="O6" s="18" t="s">
-        <v>30</v>
-      </c>
-      <c r="P6" s="18" t="s">
+    </row>
+    <row r="7" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="19"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="Q6" s="18" t="s">
+      <c r="J7" s="3" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15"/>
-      <c r="G7" s="23"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="3" t="s">
+      <c r="K7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="J7" s="3" t="s">
+      <c r="L7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="K7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="M7" s="23"/>
-      <c r="N7" s="23"/>
-      <c r="O7" s="23"/>
-      <c r="P7" s="23"/>
-      <c r="Q7" s="23"/>
+      <c r="M7" s="19"/>
+      <c r="N7" s="19"/>
+      <c r="O7" s="19"/>
+      <c r="P7" s="19"/>
+      <c r="Q7" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="O6:O7"/>
+    <mergeCell ref="P6:P7"/>
+    <mergeCell ref="Q6:Q7"/>
     <mergeCell ref="A1:Q2"/>
     <mergeCell ref="A4:A7"/>
     <mergeCell ref="B4:B7"/>
@@ -1454,9 +1504,6 @@
     <mergeCell ref="I6:L6"/>
     <mergeCell ref="M6:M7"/>
     <mergeCell ref="N6:N7"/>
-    <mergeCell ref="O6:O7"/>
-    <mergeCell ref="P6:P7"/>
-    <mergeCell ref="Q6:Q7"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1480,7 +1527,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1514,61 +1561,61 @@
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="21" t="s">
+      <c r="H3" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="I3" s="21"/>
-      <c r="J3" s="21"/>
-      <c r="K3" s="21"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
     </row>
     <row r="4" spans="1:11" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="14" t="s">
+      <c r="B4" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="14" t="s">
+      <c r="C4" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="14" t="s">
+      <c r="D4" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="14" t="s">
+      <c r="E4" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="14" t="s">
+      <c r="F4" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="20" t="s">
-        <v>42</v>
-      </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="17"/>
+      <c r="G4" s="14" t="s">
+        <v>39</v>
+      </c>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
     </row>
     <row r="5" spans="1:11" ht="30.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
       <c r="G5" s="4" t="s">
         <v>8</v>
       </c>
       <c r="H5" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K5" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="J5" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="K5" s="4" t="s">
-        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1589,6 +1636,214 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A747F49-C3F9-43FD-9F7C-32924351C960}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:O6"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.58203125" customWidth="1"/>
+    <col min="2" max="2" width="10.58203125" customWidth="1"/>
+    <col min="3" max="3" width="20.58203125" customWidth="1"/>
+    <col min="4" max="15" width="8.58203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
+      <c r="L1" s="24"/>
+      <c r="M1" s="24"/>
+      <c r="N1" s="24"/>
+      <c r="O1" s="24"/>
+    </row>
+    <row r="2" spans="1:15" ht="20" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="24"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
+      <c r="I2" s="24"/>
+      <c r="J2" s="24"/>
+      <c r="K2" s="24"/>
+      <c r="L2" s="24"/>
+      <c r="M2" s="24"/>
+      <c r="N2" s="24"/>
+      <c r="O2" s="24"/>
+    </row>
+    <row r="3" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="25"/>
+      <c r="I3" s="25"/>
+      <c r="J3" s="25"/>
+      <c r="K3" s="25"/>
+      <c r="L3" s="25"/>
+      <c r="M3" s="25"/>
+      <c r="N3" s="25"/>
+      <c r="O3" s="25"/>
+    </row>
+    <row r="4" spans="1:15" ht="32" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="26" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="C4" s="26"/>
+      <c r="D4" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="26"/>
+      <c r="F4" s="26" t="s">
+        <v>96</v>
+      </c>
+      <c r="G4" s="26"/>
+      <c r="H4" s="26" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="26"/>
+      <c r="J4" s="26" t="s">
+        <v>97</v>
+      </c>
+      <c r="K4" s="26"/>
+      <c r="L4" s="26" t="s">
+        <v>98</v>
+      </c>
+      <c r="M4" s="26"/>
+      <c r="N4" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="O4" s="26"/>
+    </row>
+    <row r="5" spans="1:15" ht="22" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="26"/>
+      <c r="B5" s="26"/>
+      <c r="C5" s="26"/>
+      <c r="D5" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="E5" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="F5" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="G5" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="H5" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="I5" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="J5" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="K5" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="L5" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="M5" s="27" t="s">
+        <v>95</v>
+      </c>
+      <c r="N5" s="27" t="s">
+        <v>94</v>
+      </c>
+      <c r="O5" s="27" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="27">
+        <v>1</v>
+      </c>
+      <c r="B6" s="26">
+        <v>2</v>
+      </c>
+      <c r="C6" s="26"/>
+      <c r="D6" s="27">
+        <v>3</v>
+      </c>
+      <c r="E6" s="27">
+        <v>4</v>
+      </c>
+      <c r="F6" s="27">
+        <v>5</v>
+      </c>
+      <c r="G6" s="27">
+        <v>6</v>
+      </c>
+      <c r="H6" s="27">
+        <v>7</v>
+      </c>
+      <c r="I6" s="27">
+        <v>8</v>
+      </c>
+      <c r="J6" s="27">
+        <v>9</v>
+      </c>
+      <c r="K6" s="27">
+        <v>10</v>
+      </c>
+      <c r="L6" s="27">
+        <v>11</v>
+      </c>
+      <c r="M6" s="27">
+        <v>12</v>
+      </c>
+      <c r="N6" s="27">
+        <v>13</v>
+      </c>
+      <c r="O6" s="27">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="11">
+    <mergeCell ref="N4:O4"/>
+    <mergeCell ref="A1:O2"/>
+    <mergeCell ref="A3:O3"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:C5"/>
+    <mergeCell ref="B6:C6"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="F4:G4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="L4:M4"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="87" fitToHeight="0" orientation="landscape" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E02BEED-3CB0-4808-9B53-A7ED62920C07}">
   <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
@@ -1599,7 +1854,7 @@
   <sheetData>
     <row r="1" spans="1:11" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>57</v>
+        <v>90</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1622,81 +1877,81 @@
       <c r="G2" s="1"/>
       <c r="H2" s="5"/>
       <c r="I2" s="1"/>
-      <c r="J2" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="K2" s="13"/>
+      <c r="J2" s="21" t="s">
+        <v>38</v>
+      </c>
+      <c r="K2" s="22"/>
     </row>
     <row r="3" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" s="17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="12" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="13"/>
+      <c r="B4" s="20" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>47</v>
+      </c>
+      <c r="D4" s="15"/>
+      <c r="E4" s="23" t="s">
         <v>48</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="F4" s="15"/>
+      <c r="G4" s="23" t="s">
         <v>49</v>
       </c>
-      <c r="C3" s="17"/>
-      <c r="D3" s="17"/>
-      <c r="E3" s="17"/>
-      <c r="F3" s="17"/>
-      <c r="G3" s="17"/>
-      <c r="H3" s="17"/>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-      <c r="K3" s="14" t="s">
+      <c r="H4" s="15"/>
+      <c r="I4" s="23" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="4" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="15"/>
-      <c r="B4" s="18" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" s="19" t="s">
+      <c r="J4" s="15"/>
+      <c r="K4" s="13"/>
+    </row>
+    <row r="5" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="17"/>
-      <c r="E4" s="19" t="s">
+      <c r="D5" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F4" s="17"/>
-      <c r="G4" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="H4" s="17"/>
-      <c r="I4" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="J4" s="17"/>
-      <c r="K4" s="15"/>
-    </row>
-    <row r="5" spans="1:11" ht="19" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>56</v>
-      </c>
       <c r="E5" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="K5" s="15"/>
+        <v>52</v>
+      </c>
+      <c r="K5" s="13"/>
     </row>
   </sheetData>
   <mergeCells count="10">
@@ -1716,7 +1971,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D53163-EA69-4728-BC12-4022B22CFEA3}">
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
@@ -1752,7 +2007,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -1832,229 +2087,220 @@
       <c r="Q3" s="5"/>
       <c r="R3" s="7"/>
       <c r="S3" s="5"/>
-      <c r="T3" s="12" t="s">
+      <c r="T3" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="U3" s="22"/>
+      <c r="V3" s="22"/>
+      <c r="W3" s="22"/>
+      <c r="X3" s="22"/>
+      <c r="Y3" s="22"/>
+      <c r="Z3" s="22"/>
+      <c r="AA3" s="22"/>
+      <c r="AB3" s="22"/>
+    </row>
+    <row r="4" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="15"/>
+      <c r="H4" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="17" t="s">
+        <v>27</v>
+      </c>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
+      <c r="S4" s="15"/>
+      <c r="T4" s="15"/>
+      <c r="U4" s="15"/>
+      <c r="V4" s="15"/>
+      <c r="W4" s="15"/>
+      <c r="X4" s="15"/>
+      <c r="Y4" s="15"/>
+      <c r="Z4" s="15"/>
+      <c r="AA4" s="15"/>
+      <c r="AB4" s="15"/>
+    </row>
+    <row r="5" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="13"/>
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="R5" s="15"/>
+      <c r="S5" s="15"/>
+      <c r="T5" s="15"/>
+      <c r="U5" s="15"/>
+      <c r="V5" s="15"/>
+      <c r="W5" s="15"/>
+      <c r="X5" s="15"/>
+      <c r="Y5" s="15"/>
+      <c r="Z5" s="15"/>
+      <c r="AA5" s="15"/>
+      <c r="AB5" s="15"/>
+    </row>
+    <row r="6" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="R6" s="15"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="U6" s="15"/>
+      <c r="V6" s="15"/>
+      <c r="W6" s="17" t="s">
+        <v>14</v>
+      </c>
+      <c r="X6" s="15"/>
+      <c r="Y6" s="15"/>
+      <c r="Z6" s="17" t="s">
         <v>83</v>
       </c>
-      <c r="U3" s="13"/>
-      <c r="V3" s="13"/>
-      <c r="W3" s="13"/>
-      <c r="X3" s="13"/>
-      <c r="Y3" s="13"/>
-      <c r="Z3" s="13"/>
-      <c r="AA3" s="13"/>
-      <c r="AB3" s="13"/>
-    </row>
-    <row r="4" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="B4" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="16" t="s">
+      <c r="AA6" s="15"/>
+      <c r="AB6" s="15"/>
+    </row>
+    <row r="7" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="G4" s="17"/>
-      <c r="H4" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="I4" s="17"/>
-      <c r="J4" s="17"/>
-      <c r="K4" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="L4" s="17"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="17"/>
-      <c r="O4" s="17"/>
-      <c r="P4" s="17"/>
-      <c r="Q4" s="17"/>
-      <c r="R4" s="17"/>
-      <c r="S4" s="17"/>
-      <c r="T4" s="17"/>
-      <c r="U4" s="17"/>
-      <c r="V4" s="17"/>
-      <c r="W4" s="17"/>
-      <c r="X4" s="17"/>
-      <c r="Y4" s="17"/>
-      <c r="Z4" s="17"/>
-      <c r="AA4" s="17"/>
-      <c r="AB4" s="17"/>
-    </row>
-    <row r="5" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="16" t="s">
+      <c r="H7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="16" t="s">
-        <v>86</v>
-      </c>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17"/>
-      <c r="P5" s="17"/>
-      <c r="Q5" s="16" t="s">
-        <v>87</v>
-      </c>
-      <c r="R5" s="17"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="17"/>
-      <c r="U5" s="17"/>
-      <c r="V5" s="17"/>
-      <c r="W5" s="17"/>
-      <c r="X5" s="17"/>
-      <c r="Y5" s="17"/>
-      <c r="Z5" s="17"/>
-      <c r="AA5" s="17"/>
-      <c r="AB5" s="17"/>
-    </row>
-    <row r="6" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="17"/>
-      <c r="H6" s="17"/>
-      <c r="I6" s="17"/>
-      <c r="J6" s="17"/>
-      <c r="K6" s="16" t="s">
+      <c r="J7" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="L7" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="L6" s="17"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="O6" s="17"/>
-      <c r="P6" s="17"/>
-      <c r="Q6" s="16" t="s">
+      <c r="M7" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="N7" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="O7" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="R6" s="17"/>
-      <c r="S6" s="17"/>
-      <c r="T6" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="U6" s="17"/>
-      <c r="V6" s="17"/>
-      <c r="W6" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="X6" s="17"/>
-      <c r="Y6" s="17"/>
-      <c r="Z6" s="16" t="s">
-        <v>89</v>
-      </c>
-      <c r="AA6" s="17"/>
-      <c r="AB6" s="17"/>
-    </row>
-    <row r="7" spans="1:28" ht="15.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="K7" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="L7" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="M7" s="6" t="s">
-        <v>90</v>
-      </c>
-      <c r="N7" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="O7" s="6" t="s">
-        <v>91</v>
-      </c>
       <c r="P7" s="6" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Q7" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="S7" s="6" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="T7" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="U7" s="6" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="V7" s="6" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="W7" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="X7" s="6" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="Y7" s="6" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="Z7" s="6" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="AA7" s="6" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="AB7" s="6" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="H5:J6"/>
-    <mergeCell ref="K5:P5"/>
-    <mergeCell ref="Q5:AB5"/>
-    <mergeCell ref="K6:M6"/>
-    <mergeCell ref="N6:P6"/>
-    <mergeCell ref="Q6:S6"/>
-    <mergeCell ref="T6:V6"/>
-    <mergeCell ref="W6:Y6"/>
-    <mergeCell ref="Z6:AB6"/>
     <mergeCell ref="A1:AB2"/>
     <mergeCell ref="T3:AB3"/>
     <mergeCell ref="A4:A7"/>
@@ -2065,6 +2311,15 @@
     <mergeCell ref="F4:G6"/>
     <mergeCell ref="H4:J4"/>
     <mergeCell ref="K4:AB4"/>
+    <mergeCell ref="H5:J6"/>
+    <mergeCell ref="K5:P5"/>
+    <mergeCell ref="Q5:AB5"/>
+    <mergeCell ref="K6:M6"/>
+    <mergeCell ref="N6:P6"/>
+    <mergeCell ref="Q6:S6"/>
+    <mergeCell ref="T6:V6"/>
+    <mergeCell ref="W6:Y6"/>
+    <mergeCell ref="Z6:AB6"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2072,7 +2327,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{82FAAEAC-4E30-4DFF-B50F-4452B5A88A25}">
   <dimension ref="A1:AB3"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
@@ -2106,7 +2361,7 @@
   <sheetData>
     <row r="1" spans="1:28" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="10" t="s">
-        <v>82</v>
+        <v>92</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2171,85 +2426,85 @@
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="H3" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="I3" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="E3" s="9" t="s">
+      <c r="J3" s="9" t="s">
         <v>61</v>
-      </c>
-      <c r="F3" s="9" t="s">
-        <v>62</v>
-      </c>
-      <c r="G3" s="9" t="s">
-        <v>63</v>
-      </c>
-      <c r="H3" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="I3" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="J3" s="9" t="s">
-        <v>66</v>
       </c>
       <c r="K3" s="9" t="s">
         <v>6</v>
       </c>
       <c r="L3" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="M3" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="N3" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="O3" s="9" t="s">
+        <v>64</v>
+      </c>
+      <c r="P3" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="Q3" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="R3" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="M3" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="N3" s="9" t="s">
+      <c r="S3" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="O3" s="9" t="s">
+      <c r="T3" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="P3" s="9" t="s">
+      <c r="U3" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="Q3" s="9" t="s">
+      <c r="V3" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="R3" s="9" t="s">
+      <c r="W3" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="S3" s="9" t="s">
+      <c r="X3" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="T3" s="9" t="s">
+      <c r="Y3" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="U3" s="9" t="s">
+      <c r="Z3" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="V3" s="9" t="s">
+      <c r="AA3" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="W3" s="9" t="s">
-        <v>77</v>
-      </c>
-      <c r="X3" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="Y3" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="Z3" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="AA3" s="9" t="s">
-        <v>81</v>
-      </c>
       <c r="AB3" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>